<commit_message>
Update forecast data 2026-09-08_20-37-20
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B941"/>
+  <dimension ref="A1:B942"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7917,6 +7917,14 @@
         <v>4.83103</v>
       </c>
     </row>
+    <row r="942" spans="1:2">
+      <c r="A942" s="3">
+        <v>46276</v>
+      </c>
+      <c r="B942">
+        <v>4.84069</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-09-15_21-02-23
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B942"/>
+  <dimension ref="A1:B943"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7925,6 +7925,14 @@
         <v>4.80765</v>
       </c>
     </row>
+    <row r="943" spans="1:2">
+      <c r="A943" s="3">
+        <v>46283</v>
+      </c>
+      <c r="B943">
+        <v>4.78793</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-09-22_20-36-35
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B943"/>
+  <dimension ref="A1:B944"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7933,6 +7933,14 @@
         <v>4.7644</v>
       </c>
     </row>
+    <row r="944" spans="1:2">
+      <c r="A944" s="3">
+        <v>46290</v>
+      </c>
+      <c r="B944">
+        <v>4.76171</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-09-29_20-35-34
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B944"/>
+  <dimension ref="A1:B945"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7941,6 +7941,14 @@
         <v>4.72135</v>
       </c>
     </row>
+    <row r="945" spans="1:2">
+      <c r="A945" s="3">
+        <v>46297</v>
+      </c>
+      <c r="B945">
+        <v>4.70822</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-10-07_18-42-59
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B945"/>
+  <dimension ref="A1:B946"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7949,6 +7949,14 @@
         <v>4.66275</v>
       </c>
     </row>
+    <row r="946" spans="1:2">
+      <c r="A946" s="3">
+        <v>46304</v>
+      </c>
+      <c r="B946">
+        <v>4.67878</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-10-13_20-34-34
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B946"/>
+  <dimension ref="A1:B947"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7957,6 +7957,14 @@
         <v>4.67727</v>
       </c>
     </row>
+    <row r="947" spans="1:2">
+      <c r="A947" s="3">
+        <v>46311</v>
+      </c>
+      <c r="B947">
+        <v>4.65983</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish fixed-origin weekly forecasts and isolated evidence
Migrate all ten symbols to completed-week origins and the current decision chain. Distinguish legacy replay, unique-week evidence, and uncalibrated reference bands; refresh client cache keys.
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B947"/>
+  <dimension ref="A1:B946"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7957,14 +7957,6 @@
         <v>4.67727</v>
       </c>
     </row>
-    <row r="947" spans="1:2">
-      <c r="A947" s="3">
-        <v>46311</v>
-      </c>
-      <c r="B947">
-        <v>4.67508</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forecast data 2026-10-15_20-34-14
</commit_message>
<xml_diff>
--- a/public/data/files/AUDCNH_diff_0th_diff.xlsx
+++ b/public/data/files/AUDCNH_diff_0th_diff.xlsx
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B946"/>
+  <dimension ref="A1:B947"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -7957,6 +7957,14 @@
         <v>4.67727</v>
       </c>
     </row>
+    <row r="947" spans="1:2">
+      <c r="A947" s="3">
+        <v>46311</v>
+      </c>
+      <c r="B947">
+        <v>4.67072</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>